<commit_message>
update data package at: 2026-09-29T15:03:51
</commit_message>
<xml_diff>
--- a/data/BASE_LIMITE_COTA.xlsx
+++ b/data/BASE_LIMITE_COTA.xlsx
@@ -977,7 +977,7 @@
         <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>8846022621</v>
+        <v>7693883880</v>
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
@@ -1010,7 +1010,7 @@
         <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>1073299042</v>
+        <v>591808934</v>
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
@@ -3221,7 +3221,7 @@
         <v>0</v>
       </c>
       <c r="G84" t="n">
-        <v>57609779</v>
+        <v>321325085</v>
       </c>
       <c r="H84" t="inlineStr"/>
       <c r="I84" t="inlineStr"/>
@@ -3386,7 +3386,7 @@
         <v>0</v>
       </c>
       <c r="G89" t="n">
-        <v>403</v>
+        <v>5358825</v>
       </c>
       <c r="H89" t="inlineStr"/>
       <c r="I89" t="inlineStr"/>
@@ -5531,7 +5531,7 @@
         <v>0</v>
       </c>
       <c r="G154" t="n">
-        <v>344522769</v>
+        <v>1417444807</v>
       </c>
       <c r="H154" t="inlineStr"/>
       <c r="I154" t="inlineStr"/>
@@ -5564,7 +5564,7 @@
         <v>1</v>
       </c>
       <c r="G155" t="n">
-        <v>20437117</v>
+        <v>67263520</v>
       </c>
       <c r="H155" t="inlineStr"/>
       <c r="I155" t="inlineStr"/>
@@ -5696,7 +5696,7 @@
         <v>0</v>
       </c>
       <c r="G159" t="n">
-        <v>5991404</v>
+        <v>6902123</v>
       </c>
       <c r="H159" t="inlineStr"/>
       <c r="I159" t="inlineStr"/>
@@ -6620,7 +6620,7 @@
         <v>0</v>
       </c>
       <c r="G187" t="n">
-        <v>31623085</v>
+        <v>248690525</v>
       </c>
       <c r="H187" t="inlineStr"/>
       <c r="I187" t="inlineStr"/>
@@ -6719,7 +6719,7 @@
         <v>0</v>
       </c>
       <c r="G190" t="n">
-        <v>2043669</v>
+        <v>28872190</v>
       </c>
       <c r="H190" t="inlineStr"/>
       <c r="I190" t="inlineStr"/>

</xml_diff>

<commit_message>
atualiza main com dados da versão 1
</commit_message>
<xml_diff>
--- a/data/BASE_LIMITE_COTA.xlsx
+++ b/data/BASE_LIMITE_COTA.xlsx
@@ -977,7 +977,7 @@
         <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>7693883880</v>
+        <v>8846022621</v>
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
@@ -1010,7 +1010,7 @@
         <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>591808934</v>
+        <v>1073299042</v>
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
@@ -3221,7 +3221,7 @@
         <v>0</v>
       </c>
       <c r="G84" t="n">
-        <v>321325085</v>
+        <v>57609779</v>
       </c>
       <c r="H84" t="inlineStr"/>
       <c r="I84" t="inlineStr"/>
@@ -3386,7 +3386,7 @@
         <v>0</v>
       </c>
       <c r="G89" t="n">
-        <v>5358825</v>
+        <v>403</v>
       </c>
       <c r="H89" t="inlineStr"/>
       <c r="I89" t="inlineStr"/>
@@ -5531,7 +5531,7 @@
         <v>0</v>
       </c>
       <c r="G154" t="n">
-        <v>1417444807</v>
+        <v>344522769</v>
       </c>
       <c r="H154" t="inlineStr"/>
       <c r="I154" t="inlineStr"/>
@@ -5564,7 +5564,7 @@
         <v>1</v>
       </c>
       <c r="G155" t="n">
-        <v>67263520</v>
+        <v>20437117</v>
       </c>
       <c r="H155" t="inlineStr"/>
       <c r="I155" t="inlineStr"/>
@@ -5696,7 +5696,7 @@
         <v>0</v>
       </c>
       <c r="G159" t="n">
-        <v>6902123</v>
+        <v>5991404</v>
       </c>
       <c r="H159" t="inlineStr"/>
       <c r="I159" t="inlineStr"/>
@@ -6620,7 +6620,7 @@
         <v>0</v>
       </c>
       <c r="G187" t="n">
-        <v>248690525</v>
+        <v>31623085</v>
       </c>
       <c r="H187" t="inlineStr"/>
       <c r="I187" t="inlineStr"/>
@@ -6719,7 +6719,7 @@
         <v>0</v>
       </c>
       <c r="G190" t="n">
-        <v>28872190</v>
+        <v>2043669</v>
       </c>
       <c r="H190" t="inlineStr"/>
       <c r="I190" t="inlineStr"/>

</xml_diff>